<commit_message>
Update code and dataset for VAR model
</commit_message>
<xml_diff>
--- a/esg/Economic_data sources.xlsx
+++ b/esg/Economic_data sources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/70cb1296250e4377/Documents/GitHub/rit/esg/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{427EE8D2-4FFE-468F-8B84-0B953C77B47A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6E7F4C2-0CAF-4F38-B8B9-628E97AF0CF5}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{427EE8D2-4FFE-468F-8B84-0B953C77B47A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A80FAAF-1332-4C51-BF25-485E0F38F084}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{EAA9D092-4ED2-424A-B9EB-6C7DC7123FC9}"/>
+    <workbookView xWindow="29970" yWindow="1170" windowWidth="21600" windowHeight="11055" xr2:uid="{EAA9D092-4ED2-424A-B9EB-6C7DC7123FC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="50">
   <si>
     <t xml:space="preserve">Economic Variables </t>
   </si>
@@ -151,18 +151,12 @@
     <t>$</t>
   </si>
   <si>
-    <t xml:space="preserve">Refinitiv Eikon  </t>
-  </si>
-  <si>
     <t xml:space="preserve">Unemployment rate </t>
   </si>
   <si>
     <t>NSW; seasonally adjusted</t>
   </si>
   <si>
-    <t xml:space="preserve"> Rate </t>
-  </si>
-  <si>
     <t xml:space="preserve">Monthly  </t>
   </si>
   <si>
@@ -173,6 +167,24 @@
   </si>
   <si>
     <t>Australian Dollar Trade-weighted Index</t>
+  </si>
+  <si>
+    <t>RBA F17</t>
+  </si>
+  <si>
+    <t>RBA F5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate </t>
+  </si>
+  <si>
+    <t>ABS Table 17</t>
+  </si>
+  <si>
+    <t>ABS Table 1</t>
+  </si>
+  <si>
+    <t>Yahoo Finance</t>
   </si>
 </sst>
 </file>
@@ -583,18 +595,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79FC165-2B35-461D-9B09-ED457D7BA268}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="64.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="47.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -620,7 +632,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -640,13 +652,16 @@
         <v>44498</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -666,13 +681,16 @@
         <v>44498</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -692,13 +710,16 @@
         <v>44530</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -720,7 +741,7 @@
       </c>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
@@ -742,7 +763,7 @@
       </c>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
@@ -762,13 +783,16 @@
         <v>44348</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
@@ -788,112 +812,124 @@
         <v>44440</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="2">
+        <v>33970</v>
+      </c>
+      <c r="F9" s="2">
+        <v>44520</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="1"/>
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="2">
+        <v>28522</v>
+      </c>
+      <c r="F10" s="2">
+        <v>44440</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="2">
+        <v>30651</v>
+      </c>
+      <c r="F11" s="2">
+        <v>44501</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E16" s="2">
         <v>38353</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F16" s="2">
         <v>44440</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H16" s="6" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="2">
-        <v>33970</v>
-      </c>
-      <c r="F10" s="2">
-        <v>44520</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" s="2">
-        <v>28522</v>
-      </c>
-      <c r="F11" s="2">
-        <v>44440</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="2">
-        <v>30651</v>
-      </c>
-      <c r="F12" s="2">
-        <v>44501</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -902,9 +938,9 @@
     <hyperlink ref="H8" r:id="rId2" location="data-download " xr:uid="{0663EB6D-181F-4560-806D-7BEC0E0D73B3}"/>
     <hyperlink ref="H2" r:id="rId3" display="https://www.rba.gov.au/statistics/historical-data.html" xr:uid="{E37481AC-CCE3-4A5C-B50B-98A093DACD85}"/>
     <hyperlink ref="H3" r:id="rId4" display="https://www.rba.gov.au/statistics/historical-data.html" xr:uid="{E997E7C9-400A-451A-AE4B-D0F501D0A389}"/>
-    <hyperlink ref="H11" r:id="rId5" location="data-downloads " xr:uid="{4A32129D-8280-4427-BD7E-6A6480370BC9}"/>
-    <hyperlink ref="H12" r:id="rId6" xr:uid="{368D1EBA-907E-4C9D-991B-E5EF83845CB6}"/>
-    <hyperlink ref="H9" r:id="rId7" xr:uid="{F9FF3683-E202-402D-A515-C2EAE5B003AC}"/>
+    <hyperlink ref="H10" r:id="rId5" location="data-downloads " xr:uid="{4A32129D-8280-4427-BD7E-6A6480370BC9}"/>
+    <hyperlink ref="H11" r:id="rId6" xr:uid="{368D1EBA-907E-4C9D-991B-E5EF83845CB6}"/>
+    <hyperlink ref="H16" r:id="rId7" xr:uid="{F9FF3683-E202-402D-A515-C2EAE5B003AC}"/>
     <hyperlink ref="H4" r:id="rId8" xr:uid="{DF19BB75-8A57-4D9C-97FB-719DDDC64601}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Data source changed: home value index
</commit_message>
<xml_diff>
--- a/esg/Economic_data sources.xlsx
+++ b/esg/Economic_data sources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/70cb1296250e4377/Documents/GitHub/rit/esg/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5289576_ad_unsw_edu_au/Documents/rit/esg/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{427EE8D2-4FFE-468F-8B84-0B953C77B47A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A80FAAF-1332-4C51-BF25-485E0F38F084}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{427EE8D2-4FFE-468F-8B84-0B953C77B47A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F19A5769-E040-3249-8E7E-AE9C6A48A631}"/>
   <bookViews>
-    <workbookView xWindow="29970" yWindow="1170" windowWidth="21600" windowHeight="11055" xr2:uid="{EAA9D092-4ED2-424A-B9EB-6C7DC7123FC9}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{EAA9D092-4ED2-424A-B9EB-6C7DC7123FC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="52">
   <si>
     <t xml:space="preserve">Economic Variables </t>
   </si>
@@ -106,9 +106,6 @@
     <t>coreLogic</t>
   </si>
   <si>
-    <t xml:space="preserve">Hedonic rental yields </t>
-  </si>
-  <si>
     <t>GDP per capita</t>
   </si>
   <si>
@@ -185,6 +182,15 @@
   </si>
   <si>
     <t>Yahoo Finance</t>
+  </si>
+  <si>
+    <t>https://www.macrotrends.net/3267/australia-real-home-prices</t>
+  </si>
+  <si>
+    <t>Bank for International Settlements</t>
+  </si>
+  <si>
+    <t>Hedonic rental yields (removed from data list)</t>
   </si>
 </sst>
 </file>
@@ -262,7 +268,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -278,6 +284,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -596,17 +605,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79FC165-2B35-461D-9B09-ED457D7BA268}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="47.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -632,7 +641,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -652,7 +661,7 @@
         <v>44498</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>13</v>
@@ -661,7 +670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -681,7 +690,7 @@
         <v>44498</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>13</v>
@@ -690,7 +699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -710,7 +719,7 @@
         <v>44530</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>18</v>
@@ -719,7 +728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -728,22 +737,24 @@
         <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E5" s="2">
         <v>29221</v>
       </c>
       <c r="F5" s="2">
-        <v>44317</v>
+        <v>46022</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
@@ -763,18 +774,18 @@
       </c>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="E7" s="2">
         <v>21794</v>
@@ -783,27 +794,27 @@
         <v>44348</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" s="2">
         <v>17777</v>
@@ -812,24 +823,24 @@
         <v>44440</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>11</v>
@@ -841,25 +852,25 @@
         <v>44520</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="E10" s="2">
         <v>28522</v>
@@ -868,21 +879,21 @@
         <v>44440</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>20</v>
@@ -906,12 +917,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>10</v>
@@ -942,6 +953,7 @@
     <hyperlink ref="H11" r:id="rId6" xr:uid="{368D1EBA-907E-4C9D-991B-E5EF83845CB6}"/>
     <hyperlink ref="H16" r:id="rId7" xr:uid="{F9FF3683-E202-402D-A515-C2EAE5B003AC}"/>
     <hyperlink ref="H4" r:id="rId8" xr:uid="{DF19BB75-8A57-4D9C-97FB-719DDDC64601}"/>
+    <hyperlink ref="H5" r:id="rId9" xr:uid="{DCFC2C9E-F459-A24E-A865-89737485546D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>